<commit_message>
Refactoreo en calculo de mezcla. Fix decimales y fracciones en inputs de prompts
</commit_message>
<xml_diff>
--- a/doc/calculador_insumos.xlsx
+++ b/doc/calculador_insumos.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7650" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7650"/>
   </bookViews>
   <sheets>
     <sheet name="Calculador de insumos liquidos" sheetId="1" r:id="rId1"/>
@@ -253,7 +253,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -274,19 +274,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.39997558519241921"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="8" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC000"/>
+        <fgColor theme="2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -453,7 +447,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
@@ -489,12 +483,12 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="5" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
@@ -516,13 +510,12 @@
     <xf numFmtId="43" fontId="0" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="43" fontId="0" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="43" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="43" fontId="0" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="43" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Millares" xfId="1" builtinId="3"/>
@@ -809,20 +802,23 @@
   <cols>
     <col min="1" max="1" width="27.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="4" customWidth="1"/>
     <col min="7" max="7" width="20.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="5" customWidth="1"/>
     <col min="11" max="11" width="24" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="4.28515625" customWidth="1"/>
     <col min="14" max="14" width="19.7109375" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="52" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="52" t="s">
+    <row r="1" spans="1:15" s="57" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="57" t="s">
         <v>30</v>
       </c>
-      <c r="B1" s="52" t="s">
+      <c r="B1" s="57" t="s">
         <v>39</v>
       </c>
     </row>
@@ -878,7 +874,7 @@
       </c>
       <c r="B5" s="30">
         <f>B4*SQRT(O12)</f>
-        <v>20.523157651784484</v>
+        <v>41.046315303568967</v>
       </c>
       <c r="G5" s="1" t="s">
         <v>35</v>
@@ -932,7 +928,7 @@
         <v>21</v>
       </c>
       <c r="L8" s="10">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -989,14 +985,14 @@
       </c>
       <c r="L10" s="11">
         <f>I10*1000*(L$8/H$4)</f>
-        <v>22.222222222222221</v>
+        <v>5.5555555555555554</v>
       </c>
       <c r="N10" s="4" t="s">
         <v>23</v>
       </c>
       <c r="O10" s="26">
         <f>L8</f>
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1025,7 +1021,7 @@
       </c>
       <c r="L11" s="11">
         <f t="shared" ref="L11:L14" si="0">I11*1000*(L$8/H$4)</f>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N11" s="24" t="s">
         <v>24</v>
@@ -1060,14 +1056,14 @@
       </c>
       <c r="L12" s="11">
         <f t="shared" si="0"/>
-        <v>444.44444444444446</v>
+        <v>111.11111111111111</v>
       </c>
       <c r="N12" s="1" t="s">
         <v>25</v>
       </c>
       <c r="O12" s="25">
         <f>O11/O10</f>
-        <v>1.3</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
@@ -1096,7 +1092,7 @@
       </c>
       <c r="L13" s="11">
         <f t="shared" si="0"/>
-        <v>80</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1124,14 +1120,14 @@
       </c>
       <c r="L14" s="12">
         <f t="shared" si="0"/>
-        <v>3475.5555555555561</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" s="53" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="53" t="s">
+        <v>868.88888888888903</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" s="57" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="57" t="s">
         <v>29</v>
       </c>
-      <c r="B19" s="53" t="s">
+      <c r="B19" s="57" t="s">
         <v>40</v>
       </c>
     </row>
@@ -1221,7 +1217,7 @@
       <c r="A4" t="s">
         <v>41</v>
       </c>
-      <c r="C4" s="54">
+      <c r="C4" s="52">
         <v>4</v>
       </c>
     </row>
@@ -1229,7 +1225,7 @@
       <c r="A5" t="s">
         <v>42</v>
       </c>
-      <c r="C5" s="54">
+      <c r="C5" s="52">
         <v>100</v>
       </c>
     </row>
@@ -1237,7 +1233,7 @@
       <c r="A6" t="s">
         <v>43</v>
       </c>
-      <c r="C6" s="54">
+      <c r="C6" s="52">
         <v>100</v>
       </c>
     </row>
@@ -1245,7 +1241,7 @@
       <c r="A7" t="s">
         <v>44</v>
       </c>
-      <c r="C7" s="54">
+      <c r="C7" s="52">
         <v>100</v>
       </c>
     </row>
@@ -1253,18 +1249,18 @@
       <c r="A9" t="s">
         <v>46</v>
       </c>
-      <c r="C9" s="57">
+      <c r="C9" s="55">
         <f>((C$12*(C$5/100))/(C$4))*1000000</f>
         <v>1500000</v>
       </c>
-      <c r="D9" s="55">
+      <c r="D9" s="53">
         <v>1350000</v>
       </c>
-      <c r="E9" s="58">
+      <c r="E9" s="56">
         <f>E10/(C6/100)</f>
         <v>1215000</v>
       </c>
-      <c r="F9" s="58">
+      <c r="F9" s="56">
         <f>F11/(C7/100)/(C6/100)</f>
         <v>1093500</v>
       </c>
@@ -1273,18 +1269,18 @@
       <c r="A10" t="s">
         <v>45</v>
       </c>
-      <c r="C10" s="57">
+      <c r="C10" s="55">
         <f>((C$12*(C$5/100)*(C6/100))/(C$4))*1000000</f>
         <v>1500000</v>
       </c>
-      <c r="D10" s="57">
+      <c r="D10" s="55">
         <f>D9*((C6/100))</f>
         <v>1350000</v>
       </c>
-      <c r="E10" s="56">
+      <c r="E10" s="54">
         <v>1215000</v>
       </c>
-      <c r="F10" s="58">
+      <c r="F10" s="56">
         <f>F11/(C7/100)</f>
         <v>1093500</v>
       </c>
@@ -1293,19 +1289,19 @@
       <c r="A11" t="s">
         <v>47</v>
       </c>
-      <c r="C11" s="57">
+      <c r="C11" s="55">
         <f>((C$12*(C$5/100)*(C6/100)*(C7/100))/(C$4))*1000000</f>
         <v>1500000</v>
       </c>
-      <c r="D11" s="57">
+      <c r="D11" s="55">
         <f>D9*((C6/100)*(C7/100))</f>
         <v>1350000</v>
       </c>
-      <c r="E11" s="58">
+      <c r="E11" s="56">
         <f>E10*(C7/100)</f>
         <v>1215000</v>
       </c>
-      <c r="F11" s="56">
+      <c r="F11" s="54">
         <v>1093500</v>
       </c>
     </row>
@@ -1313,18 +1309,18 @@
       <c r="A12" t="s">
         <v>48</v>
       </c>
-      <c r="C12" s="55">
+      <c r="C12" s="53">
         <v>6</v>
       </c>
-      <c r="D12" s="57">
+      <c r="D12" s="55">
         <f>((D9/1000000)*C4)/(C5/100)</f>
         <v>5.4</v>
       </c>
-      <c r="E12" s="57">
+      <c r="E12" s="55">
         <f>((E9/1000000)*C4)/(C6/100)</f>
         <v>4.8600000000000003</v>
       </c>
-      <c r="F12" s="57">
+      <c r="F12" s="55">
         <f>((F11/1000000)*C4)/((C5/100)*(C6/100)*(C7/100))</f>
         <v>4.3739999999999997</v>
       </c>

</xml_diff>